<commit_message>
fix: publish local dashboard filters and cost rules
</commit_message>
<xml_diff>
--- a/data/uploads/tongshi_demo.xlsx
+++ b/data/uploads/tongshi_demo.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="26860" windowHeight="11740"/>
+    <workbookView windowWidth="28000" windowHeight="11740"/>
   </bookViews>
   <sheets>
     <sheet name="sheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">sheet!$A$1:$Z$333</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">sheet!$A$1:$Z$352</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4056" uniqueCount="2596">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4412" uniqueCount="2796">
   <si>
     <t>日期</t>
   </si>
@@ -7818,6 +7818,606 @@
   </si>
   <si>
     <t>11343</t>
+  </si>
+  <si>
+    <t>2026-08-10</t>
+  </si>
+  <si>
+    <t>1130</t>
+  </si>
+  <si>
+    <t>0.31</t>
+  </si>
+  <si>
+    <t>72</t>
+  </si>
+  <si>
+    <t>0.00166863</t>
+  </si>
+  <si>
+    <t>46737</t>
+  </si>
+  <si>
+    <t>10188</t>
+  </si>
+  <si>
+    <t>754</t>
+  </si>
+  <si>
+    <t>643</t>
+  </si>
+  <si>
+    <t>212341</t>
+  </si>
+  <si>
+    <t>47167</t>
+  </si>
+  <si>
+    <t>11030</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>0.09</t>
+  </si>
+  <si>
+    <t>0.00455927</t>
+  </si>
+  <si>
+    <t>94074</t>
+  </si>
+  <si>
+    <t>27636</t>
+  </si>
+  <si>
+    <t>8224</t>
+  </si>
+  <si>
+    <t>4888</t>
+  </si>
+  <si>
+    <t>126</t>
+  </si>
+  <si>
+    <t>552763</t>
+  </si>
+  <si>
+    <t>239202</t>
+  </si>
+  <si>
+    <t>0.48</t>
+  </si>
+  <si>
+    <t>30456</t>
+  </si>
+  <si>
+    <t>0.00086640</t>
+  </si>
+  <si>
+    <t>361491</t>
+  </si>
+  <si>
+    <t>85411</t>
+  </si>
+  <si>
+    <t>8061</t>
+  </si>
+  <si>
+    <t>6529</t>
+  </si>
+  <si>
+    <t>74</t>
+  </si>
+  <si>
+    <t>1765600</t>
+  </si>
+  <si>
+    <t>478946</t>
+  </si>
+  <si>
+    <t>93060</t>
+  </si>
+  <si>
+    <t>188</t>
+  </si>
+  <si>
+    <t>0.29</t>
+  </si>
+  <si>
+    <t>0.00178137</t>
+  </si>
+  <si>
+    <t>214156</t>
+  </si>
+  <si>
+    <t>46032</t>
+  </si>
+  <si>
+    <t>4935</t>
+  </si>
+  <si>
+    <t>3988</t>
+  </si>
+  <si>
+    <t>82</t>
+  </si>
+  <si>
+    <t>1081194</t>
+  </si>
+  <si>
+    <t>382224</t>
+  </si>
+  <si>
+    <t>1.29</t>
+  </si>
+  <si>
+    <t>52184</t>
+  </si>
+  <si>
+    <t>0.01726593</t>
+  </si>
+  <si>
+    <t>18685</t>
+  </si>
+  <si>
+    <t>5618</t>
+  </si>
+  <si>
+    <t>2223</t>
+  </si>
+  <si>
+    <t>1363</t>
+  </si>
+  <si>
+    <t>97</t>
+  </si>
+  <si>
+    <t>162449</t>
+  </si>
+  <si>
+    <t>98896</t>
+  </si>
+  <si>
+    <t>6917</t>
+  </si>
+  <si>
+    <t>0.00177368</t>
+  </si>
+  <si>
+    <t>68079</t>
+  </si>
+  <si>
+    <t>16914</t>
+  </si>
+  <si>
+    <t>710</t>
+  </si>
+  <si>
+    <t>313298</t>
+  </si>
+  <si>
+    <t>55859</t>
+  </si>
+  <si>
+    <t>18025</t>
+  </si>
+  <si>
+    <t>2026-08-12</t>
+  </si>
+  <si>
+    <t>0.00230428</t>
+  </si>
+  <si>
+    <t>469489</t>
+  </si>
+  <si>
+    <t>121079</t>
+  </si>
+  <si>
+    <t>25118</t>
+  </si>
+  <si>
+    <t>17983</t>
+  </si>
+  <si>
+    <t>279</t>
+  </si>
+  <si>
+    <t>2913673</t>
+  </si>
+  <si>
+    <t>1223437</t>
+  </si>
+  <si>
+    <t>138097</t>
+  </si>
+  <si>
+    <t>0.00074264</t>
+  </si>
+  <si>
+    <t>743312</t>
+  </si>
+  <si>
+    <t>195249</t>
+  </si>
+  <si>
+    <t>19908</t>
+  </si>
+  <si>
+    <t>16480</t>
+  </si>
+  <si>
+    <t>4240465</t>
+  </si>
+  <si>
+    <t>1163770</t>
+  </si>
+  <si>
+    <t>214580</t>
+  </si>
+  <si>
+    <t>0.00472740</t>
+  </si>
+  <si>
+    <t>205145</t>
+  </si>
+  <si>
+    <t>57960</t>
+  </si>
+  <si>
+    <t>13626</t>
+  </si>
+  <si>
+    <t>9334</t>
+  </si>
+  <si>
+    <t>274</t>
+  </si>
+  <si>
+    <t>1254303</t>
+  </si>
+  <si>
+    <t>503013</t>
+  </si>
+  <si>
+    <t>64439</t>
+  </si>
+  <si>
+    <t>0.00085397</t>
+  </si>
+  <si>
+    <t>154217</t>
+  </si>
+  <si>
+    <t>51524</t>
+  </si>
+  <si>
+    <t>3307</t>
+  </si>
+  <si>
+    <t>2801</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>1024172</t>
+  </si>
+  <si>
+    <t>159160</t>
+  </si>
+  <si>
+    <t>54967</t>
+  </si>
+  <si>
+    <t>0.00551861</t>
+  </si>
+  <si>
+    <t>175894</t>
+  </si>
+  <si>
+    <t>35335</t>
+  </si>
+  <si>
+    <t>10831</t>
+  </si>
+  <si>
+    <t>7383</t>
+  </si>
+  <si>
+    <t>195</t>
+  </si>
+  <si>
+    <t>1039132</t>
+  </si>
+  <si>
+    <t>604271</t>
+  </si>
+  <si>
+    <t>43659</t>
+  </si>
+  <si>
+    <t>0.01804024</t>
+  </si>
+  <si>
+    <t>64457</t>
+  </si>
+  <si>
+    <t>20676</t>
+  </si>
+  <si>
+    <t>8093</t>
+  </si>
+  <si>
+    <t>5429</t>
+  </si>
+  <si>
+    <t>373</t>
+  </si>
+  <si>
+    <t>633974</t>
+  </si>
+  <si>
+    <t>395182</t>
+  </si>
+  <si>
+    <t>25866</t>
+  </si>
+  <si>
+    <t>0.00190375</t>
+  </si>
+  <si>
+    <t>192864</t>
+  </si>
+  <si>
+    <t>56205</t>
+  </si>
+  <si>
+    <t>2969</t>
+  </si>
+  <si>
+    <t>2582</t>
+  </si>
+  <si>
+    <t>107</t>
+  </si>
+  <si>
+    <t>1092150</t>
+  </si>
+  <si>
+    <t>183219</t>
+  </si>
+  <si>
+    <t>59921</t>
+  </si>
+  <si>
+    <t>2026-08-13</t>
+  </si>
+  <si>
+    <t>0.00304233</t>
+  </si>
+  <si>
+    <t>432304</t>
+  </si>
+  <si>
+    <t>105840</t>
+  </si>
+  <si>
+    <t>26735</t>
+  </si>
+  <si>
+    <t>18736</t>
+  </si>
+  <si>
+    <t>2666715</t>
+  </si>
+  <si>
+    <t>1265835</t>
+  </si>
+  <si>
+    <t>122904</t>
+  </si>
+  <si>
+    <t>0.45</t>
+  </si>
+  <si>
+    <t>0.00100737</t>
+  </si>
+  <si>
+    <t>566542</t>
+  </si>
+  <si>
+    <t>139968</t>
+  </si>
+  <si>
+    <t>12312</t>
+  </si>
+  <si>
+    <t>10120</t>
+  </si>
+  <si>
+    <t>141</t>
+  </si>
+  <si>
+    <t>2981253</t>
+  </si>
+  <si>
+    <t>806093</t>
+  </si>
+  <si>
+    <t>153821</t>
+  </si>
+  <si>
+    <t>0.00813421</t>
+  </si>
+  <si>
+    <t>3714</t>
+  </si>
+  <si>
+    <t>1967</t>
+  </si>
+  <si>
+    <t>1022</t>
+  </si>
+  <si>
+    <t>846</t>
+  </si>
+  <si>
+    <t>55014</t>
+  </si>
+  <si>
+    <t>34469</t>
+  </si>
+  <si>
+    <t>2320</t>
+  </si>
+  <si>
+    <t>0.00088210</t>
+  </si>
+  <si>
+    <t>108689</t>
+  </si>
+  <si>
+    <t>26074</t>
+  </si>
+  <si>
+    <t>1618</t>
+  </si>
+  <si>
+    <t>1380</t>
+  </si>
+  <si>
+    <t>496055</t>
+  </si>
+  <si>
+    <t>87536</t>
+  </si>
+  <si>
+    <t>27761</t>
+  </si>
+  <si>
+    <t>0.00672665</t>
+  </si>
+  <si>
+    <t>133257</t>
+  </si>
+  <si>
+    <t>23786</t>
+  </si>
+  <si>
+    <t>8287</t>
+  </si>
+  <si>
+    <t>5686</t>
+  </si>
+  <si>
+    <t>786677</t>
+  </si>
+  <si>
+    <t>507587</t>
+  </si>
+  <si>
+    <t>30838</t>
+  </si>
+  <si>
+    <t>0.00459141</t>
+  </si>
+  <si>
+    <t>293769</t>
+  </si>
+  <si>
+    <t>88426</t>
+  </si>
+  <si>
+    <t>18581</t>
+  </si>
+  <si>
+    <t>12423</t>
+  </si>
+  <si>
+    <t>406</t>
+  </si>
+  <si>
+    <t>1850595</t>
+  </si>
+  <si>
+    <t>726084</t>
+  </si>
+  <si>
+    <t>98052</t>
+  </si>
+  <si>
+    <t>0.02077890</t>
+  </si>
+  <si>
+    <t>108174</t>
+  </si>
+  <si>
+    <t>32533</t>
+  </si>
+  <si>
+    <t>10981</t>
+  </si>
+  <si>
+    <t>7583</t>
+  </si>
+  <si>
+    <t>676</t>
+  </si>
+  <si>
+    <t>1079653</t>
+  </si>
+  <si>
+    <t>675233</t>
+  </si>
+  <si>
+    <t>42056</t>
+  </si>
+  <si>
+    <t>0.04736842</t>
+  </si>
+  <si>
+    <t>1272</t>
+  </si>
+  <si>
+    <t>570</t>
+  </si>
+  <si>
+    <t>324</t>
+  </si>
+  <si>
+    <t>29181</t>
+  </si>
+  <si>
+    <t>22551</t>
+  </si>
+  <si>
+    <t>880</t>
+  </si>
+  <si>
+    <t>0.00123097</t>
+  </si>
+  <si>
+    <t>214475</t>
+  </si>
+  <si>
+    <t>57678</t>
+  </si>
+  <si>
+    <t>3125</t>
+  </si>
+  <si>
+    <t>2734</t>
+  </si>
+  <si>
+    <t>1070946</t>
+  </si>
+  <si>
+    <t>177236</t>
+  </si>
+  <si>
+    <t>61251</t>
   </si>
 </sst>
 </file>
@@ -7839,15 +8439,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <sz val="1"/>
+      <color rgb="FFFFFFFF"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="1"/>
-      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -8445,11 +9045,13 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -8833,7 +9435,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:Z352"/>
+  <dimension ref="A1:Z387"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="16.0192307692308" style="1" customWidth="1"/>
@@ -10619,7 +11221,6 @@
       <c r="C44" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D44" s="1"/>
       <c r="E44" s="1" t="s">
         <v>25</v>
       </c>
@@ -10641,7 +11242,6 @@
       <c r="K44" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L44" s="1"/>
       <c r="M44" s="1" t="s">
         <v>26</v>
       </c>
@@ -12935,7 +13535,6 @@
       <c r="K100" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L100" s="1"/>
       <c r="M100" s="1" t="s">
         <v>157</v>
       </c>
@@ -13876,7 +14475,6 @@
       <c r="K123" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L123" s="1"/>
       <c r="M123" s="1" t="s">
         <v>149</v>
       </c>
@@ -14366,7 +14964,6 @@
       <c r="K135" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L135" s="1"/>
       <c r="M135" s="1" t="s">
         <v>364</v>
       </c>
@@ -14668,7 +15265,6 @@
       <c r="C143" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D143" s="1"/>
       <c r="E143" s="1" t="s">
         <v>262</v>
       </c>
@@ -14690,7 +15286,6 @@
       <c r="K143" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L143" s="1"/>
       <c r="M143" s="1" t="s">
         <v>26</v>
       </c>
@@ -16167,7 +16762,6 @@
       <c r="K179" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L179" s="1"/>
       <c r="M179" s="1" t="s">
         <v>1219</v>
       </c>
@@ -20962,7 +21556,6 @@
       <c r="K296" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="L296" s="1"/>
       <c r="M296" s="1" t="s">
         <v>1219</v>
       </c>
@@ -23261,20 +23854,1455 @@
         <v>2595</v>
       </c>
     </row>
+    <row r="353" spans="1:13">
+      <c r="A353" s="4" t="s">
+        <v>2596</v>
+      </c>
+      <c r="B353" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C353" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D353" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="E353" s="4" t="s">
+        <v>2190</v>
+      </c>
+      <c r="F353" s="4" t="s">
+        <v>1573</v>
+      </c>
+      <c r="G353" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="H353" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="I353" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J353" s="4" t="s">
+        <v>2597</v>
+      </c>
+      <c r="K353" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="L353" s="4" t="s">
+        <v>2598</v>
+      </c>
+      <c r="M353" s="4" t="s">
+        <v>2599</v>
+      </c>
+    </row>
+    <row r="354" spans="1:13">
+      <c r="A354" s="4" t="s">
+        <v>2596</v>
+      </c>
+      <c r="B354" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C354" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D354" s="4" t="s">
+        <v>2600</v>
+      </c>
+      <c r="E354" s="4" t="s">
+        <v>2601</v>
+      </c>
+      <c r="F354" s="4" t="s">
+        <v>2602</v>
+      </c>
+      <c r="G354" s="4" t="s">
+        <v>2603</v>
+      </c>
+      <c r="H354" s="4" t="s">
+        <v>2604</v>
+      </c>
+      <c r="I354" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="J354" s="4" t="s">
+        <v>2605</v>
+      </c>
+      <c r="K354" s="4" t="s">
+        <v>2606</v>
+      </c>
+      <c r="L354" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="M354" s="4" t="s">
+        <v>2607</v>
+      </c>
+    </row>
+    <row r="355" spans="1:13">
+      <c r="A355" s="4" t="s">
+        <v>2596</v>
+      </c>
+      <c r="B355" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C355" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D355" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="E355" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="F355" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="G355" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="H355" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="I355" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J355" s="4" t="s">
+        <v>675</v>
+      </c>
+      <c r="K355" s="4" t="s">
+        <v>2608</v>
+      </c>
+      <c r="L355" s="4" t="s">
+        <v>2609</v>
+      </c>
+      <c r="M355" s="4" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="356" spans="1:13">
+      <c r="A356" s="4" t="s">
+        <v>2596</v>
+      </c>
+      <c r="B356" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C356" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D356" s="4" t="s">
+        <v>2610</v>
+      </c>
+      <c r="E356" s="4" t="s">
+        <v>2611</v>
+      </c>
+      <c r="F356" s="4" t="s">
+        <v>2612</v>
+      </c>
+      <c r="G356" s="4" t="s">
+        <v>2613</v>
+      </c>
+      <c r="H356" s="4" t="s">
+        <v>2614</v>
+      </c>
+      <c r="I356" s="4" t="s">
+        <v>2615</v>
+      </c>
+      <c r="J356" s="4" t="s">
+        <v>2616</v>
+      </c>
+      <c r="K356" s="4" t="s">
+        <v>2617</v>
+      </c>
+      <c r="L356" s="4" t="s">
+        <v>2618</v>
+      </c>
+      <c r="M356" s="4" t="s">
+        <v>2619</v>
+      </c>
+    </row>
+    <row r="357" spans="1:13">
+      <c r="A357" s="4" t="s">
+        <v>2596</v>
+      </c>
+      <c r="B357" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C357" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D357" s="4" t="s">
+        <v>2620</v>
+      </c>
+      <c r="E357" s="4" t="s">
+        <v>2621</v>
+      </c>
+      <c r="F357" s="4" t="s">
+        <v>2622</v>
+      </c>
+      <c r="G357" s="4" t="s">
+        <v>2623</v>
+      </c>
+      <c r="H357" s="4" t="s">
+        <v>2624</v>
+      </c>
+      <c r="I357" s="4" t="s">
+        <v>2625</v>
+      </c>
+      <c r="J357" s="4" t="s">
+        <v>2626</v>
+      </c>
+      <c r="K357" s="4" t="s">
+        <v>2627</v>
+      </c>
+      <c r="L357" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="M357" s="4" t="s">
+        <v>2628</v>
+      </c>
+    </row>
+    <row r="358" spans="1:13">
+      <c r="A358" s="4" t="s">
+        <v>2596</v>
+      </c>
+      <c r="B358" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C358" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D358" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="E358" s="4" t="s">
+        <v>953</v>
+      </c>
+      <c r="F358" s="4" t="s">
+        <v>2608</v>
+      </c>
+      <c r="G358" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="H358" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="I358" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J358" s="4" t="s">
+        <v>2629</v>
+      </c>
+      <c r="K358" s="4" t="s">
+        <v>2559</v>
+      </c>
+      <c r="L358" s="4" t="s">
+        <v>2630</v>
+      </c>
+      <c r="M358" s="4" t="s">
+        <v>2608</v>
+      </c>
+    </row>
+    <row r="359" spans="1:13">
+      <c r="A359" s="4" t="s">
+        <v>2596</v>
+      </c>
+      <c r="B359" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C359" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D359" s="4" t="s">
+        <v>2631</v>
+      </c>
+      <c r="E359" s="4" t="s">
+        <v>2632</v>
+      </c>
+      <c r="F359" s="4" t="s">
+        <v>2633</v>
+      </c>
+      <c r="G359" s="4" t="s">
+        <v>2634</v>
+      </c>
+      <c r="H359" s="4" t="s">
+        <v>2635</v>
+      </c>
+      <c r="I359" s="4" t="s">
+        <v>2636</v>
+      </c>
+      <c r="J359" s="4" t="s">
+        <v>2637</v>
+      </c>
+      <c r="K359" s="4" t="s">
+        <v>2638</v>
+      </c>
+      <c r="L359" s="4" t="s">
+        <v>2639</v>
+      </c>
+      <c r="M359" s="4" t="s">
+        <v>2640</v>
+      </c>
+    </row>
+    <row r="360" spans="1:13">
+      <c r="A360" s="4" t="s">
+        <v>2596</v>
+      </c>
+      <c r="B360" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C360" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D360" s="4" t="s">
+        <v>2641</v>
+      </c>
+      <c r="E360" s="4" t="s">
+        <v>2642</v>
+      </c>
+      <c r="F360" s="4" t="s">
+        <v>2643</v>
+      </c>
+      <c r="G360" s="4" t="s">
+        <v>2644</v>
+      </c>
+      <c r="H360" s="4" t="s">
+        <v>2645</v>
+      </c>
+      <c r="I360" s="4" t="s">
+        <v>2646</v>
+      </c>
+      <c r="J360" s="4" t="s">
+        <v>2647</v>
+      </c>
+      <c r="K360" s="4" t="s">
+        <v>2648</v>
+      </c>
+      <c r="L360" s="4" t="s">
+        <v>1130</v>
+      </c>
+      <c r="M360" s="4" t="s">
+        <v>2649</v>
+      </c>
+    </row>
+    <row r="361" spans="1:13">
+      <c r="A361" s="4" t="s">
+        <v>2596</v>
+      </c>
+      <c r="B361" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C361" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D361" s="4" t="s">
+        <v>2650</v>
+      </c>
+      <c r="E361" s="4" t="s">
+        <v>2651</v>
+      </c>
+      <c r="F361" s="4" t="s">
+        <v>2652</v>
+      </c>
+      <c r="G361" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="H361" s="4" t="s">
+        <v>2653</v>
+      </c>
+      <c r="I361" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="J361" s="4" t="s">
+        <v>2654</v>
+      </c>
+      <c r="K361" s="4" t="s">
+        <v>2655</v>
+      </c>
+      <c r="L361" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="M361" s="4" t="s">
+        <v>2656</v>
+      </c>
+    </row>
+    <row r="362" spans="1:13">
+      <c r="A362" s="5">
+        <v>46245</v>
+      </c>
+      <c r="B362" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C362" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D362" s="1">
+        <v>0.00334165</v>
+      </c>
+      <c r="E362" s="1">
+        <v>302768</v>
+      </c>
+      <c r="F362" s="1">
+        <v>72120</v>
+      </c>
+      <c r="G362" s="1">
+        <v>20279</v>
+      </c>
+      <c r="H362" s="1">
+        <v>14107</v>
+      </c>
+      <c r="I362" s="1">
+        <v>241</v>
+      </c>
+      <c r="J362" s="1">
+        <v>1879967</v>
+      </c>
+      <c r="K362" s="1">
+        <v>940101</v>
+      </c>
+      <c r="L362" s="1">
+        <v>0.77</v>
+      </c>
+      <c r="M362" s="1">
+        <v>84502</v>
+      </c>
+    </row>
+    <row r="363" spans="1:13">
+      <c r="A363" s="5">
+        <v>46245</v>
+      </c>
+      <c r="B363" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C363" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D363" s="1">
+        <v>0.00122588</v>
+      </c>
+      <c r="E363" s="1">
+        <v>127821</v>
+      </c>
+      <c r="F363" s="1">
+        <v>34261</v>
+      </c>
+      <c r="G363" s="1">
+        <v>2523</v>
+      </c>
+      <c r="H363" s="1">
+        <v>2112</v>
+      </c>
+      <c r="I363" s="1">
+        <v>42</v>
+      </c>
+      <c r="J363" s="1">
+        <v>706552</v>
+      </c>
+      <c r="K363" s="1">
+        <v>125712</v>
+      </c>
+      <c r="L363" s="1">
+        <v>0.83</v>
+      </c>
+      <c r="M363" s="1">
+        <v>36748</v>
+      </c>
+    </row>
+    <row r="364" spans="1:13">
+      <c r="A364" s="5">
+        <v>46245</v>
+      </c>
+      <c r="B364" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C364" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D364" s="1">
+        <v>0.00068393</v>
+      </c>
+      <c r="E364" s="1">
+        <v>827314</v>
+      </c>
+      <c r="F364" s="1">
+        <v>214934</v>
+      </c>
+      <c r="G364" s="1">
+        <v>18087</v>
+      </c>
+      <c r="H364" s="1">
+        <v>15040</v>
+      </c>
+      <c r="I364" s="1">
+        <v>147</v>
+      </c>
+      <c r="J364" s="1">
+        <v>4533896</v>
+      </c>
+      <c r="K364" s="1">
+        <v>1061952</v>
+      </c>
+      <c r="L364" s="1">
+        <v>0.98</v>
+      </c>
+      <c r="M364" s="1">
+        <v>233544</v>
+      </c>
+    </row>
+    <row r="365" spans="1:13">
+      <c r="A365" s="5">
+        <v>46245</v>
+      </c>
+      <c r="B365" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C365" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D365" s="1">
+        <v>0.00623557</v>
+      </c>
+      <c r="E365" s="1">
+        <v>142231</v>
+      </c>
+      <c r="F365" s="1">
+        <v>25980</v>
+      </c>
+      <c r="G365" s="1">
+        <v>10201</v>
+      </c>
+      <c r="H365" s="1">
+        <v>6689</v>
+      </c>
+      <c r="I365" s="1">
+        <v>162</v>
+      </c>
+      <c r="J365" s="1">
+        <v>840225</v>
+      </c>
+      <c r="K365" s="1">
+        <v>546831</v>
+      </c>
+      <c r="L365" s="1">
+        <v>0.89</v>
+      </c>
+      <c r="M365" s="1">
+        <v>33338</v>
+      </c>
+    </row>
+    <row r="366" spans="1:13">
+      <c r="A366" s="5">
+        <v>46245</v>
+      </c>
+      <c r="B366" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C366" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D366" s="1">
+        <v>0.00546271</v>
+      </c>
+      <c r="E366" s="1">
+        <v>84915</v>
+      </c>
+      <c r="F366" s="1">
+        <v>21601</v>
+      </c>
+      <c r="G366" s="1">
+        <v>6788</v>
+      </c>
+      <c r="H366" s="1">
+        <v>4271</v>
+      </c>
+      <c r="I366" s="1">
+        <v>118</v>
+      </c>
+      <c r="J366" s="1">
+        <v>481789</v>
+      </c>
+      <c r="K366" s="1">
+        <v>228486</v>
+      </c>
+      <c r="L366" s="1">
+        <v>0.56</v>
+      </c>
+      <c r="M366" s="1">
+        <v>24434</v>
+      </c>
+    </row>
+    <row r="367" spans="1:13">
+      <c r="A367" s="5">
+        <v>46245</v>
+      </c>
+      <c r="B367" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C367" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D367" s="1">
+        <v>0.00101696</v>
+      </c>
+      <c r="E367" s="1">
+        <v>112031</v>
+      </c>
+      <c r="F367" s="1">
+        <v>24583</v>
+      </c>
+      <c r="G367" s="1">
+        <v>2464</v>
+      </c>
+      <c r="H367" s="1">
+        <v>1995</v>
+      </c>
+      <c r="I367" s="1">
+        <v>25</v>
+      </c>
+      <c r="J367" s="1">
+        <v>547891</v>
+      </c>
+      <c r="K367" s="1">
+        <v>159631</v>
+      </c>
+      <c r="L367" s="1">
+        <v>1.08</v>
+      </c>
+      <c r="M367" s="1">
+        <v>27253</v>
+      </c>
+    </row>
+    <row r="368" spans="1:13">
+      <c r="A368" s="5">
+        <v>46245</v>
+      </c>
+      <c r="B368" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C368" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D368" s="1">
+        <v>0.00994654</v>
+      </c>
+      <c r="E368" s="1">
+        <v>50139</v>
+      </c>
+      <c r="F368" s="1">
+        <v>8043</v>
+      </c>
+      <c r="G368" s="1">
+        <v>2608</v>
+      </c>
+      <c r="H368" s="1">
+        <v>1900</v>
+      </c>
+      <c r="I368" s="1">
+        <v>80</v>
+      </c>
+      <c r="J368" s="1">
+        <v>333355</v>
+      </c>
+      <c r="K368" s="1">
+        <v>229435</v>
+      </c>
+      <c r="L368" s="1">
+        <v>1.47</v>
+      </c>
+      <c r="M368" s="1">
+        <v>11433</v>
+      </c>
+    </row>
+    <row r="369" spans="1:13">
+      <c r="A369" s="5">
+        <v>46245</v>
+      </c>
+      <c r="B369" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C369" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D369" s="1">
+        <v>0.00183917</v>
+      </c>
+      <c r="E369" s="1">
+        <v>197667</v>
+      </c>
+      <c r="F369" s="1">
+        <v>58722</v>
+      </c>
+      <c r="G369" s="1">
+        <v>3329</v>
+      </c>
+      <c r="H369" s="1">
+        <v>2876</v>
+      </c>
+      <c r="I369" s="1">
+        <v>108</v>
+      </c>
+      <c r="J369" s="1">
+        <v>1137826</v>
+      </c>
+      <c r="K369" s="1">
+        <v>209398</v>
+      </c>
+      <c r="L369" s="1">
+        <v>1.05</v>
+      </c>
+      <c r="M369" s="1">
+        <v>62864</v>
+      </c>
+    </row>
+    <row r="370" spans="1:13">
+      <c r="A370" s="5">
+        <v>46245</v>
+      </c>
+      <c r="B370" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C370" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D370" s="1">
+        <v>0.01946654</v>
+      </c>
+      <c r="E370" s="1">
+        <v>92913</v>
+      </c>
+      <c r="F370" s="1">
+        <v>34829</v>
+      </c>
+      <c r="G370" s="1">
+        <v>14822</v>
+      </c>
+      <c r="H370" s="1">
+        <v>9475</v>
+      </c>
+      <c r="I370" s="1">
+        <v>678</v>
+      </c>
+      <c r="J370" s="1">
+        <v>1083922</v>
+      </c>
+      <c r="K370" s="1">
+        <v>692548</v>
+      </c>
+      <c r="L370" s="1">
+        <v>0.78</v>
+      </c>
+      <c r="M370" s="1">
+        <v>43938</v>
+      </c>
+    </row>
+    <row r="371" spans="1:13">
+      <c r="A371" s="4" t="s">
+        <v>2657</v>
+      </c>
+      <c r="B371" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C371" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D371" s="4" t="s">
+        <v>2658</v>
+      </c>
+      <c r="E371" s="4" t="s">
+        <v>2659</v>
+      </c>
+      <c r="F371" s="4" t="s">
+        <v>2660</v>
+      </c>
+      <c r="G371" s="4" t="s">
+        <v>2661</v>
+      </c>
+      <c r="H371" s="4" t="s">
+        <v>2662</v>
+      </c>
+      <c r="I371" s="4" t="s">
+        <v>2663</v>
+      </c>
+      <c r="J371" s="4" t="s">
+        <v>2664</v>
+      </c>
+      <c r="K371" s="4" t="s">
+        <v>2665</v>
+      </c>
+      <c r="L371" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="M371" s="4" t="s">
+        <v>2666</v>
+      </c>
+    </row>
+    <row r="372" spans="1:13">
+      <c r="A372" s="4" t="s">
+        <v>2657</v>
+      </c>
+      <c r="B372" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C372" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D372" s="4" t="s">
+        <v>2667</v>
+      </c>
+      <c r="E372" s="4" t="s">
+        <v>2668</v>
+      </c>
+      <c r="F372" s="4" t="s">
+        <v>2669</v>
+      </c>
+      <c r="G372" s="4" t="s">
+        <v>2670</v>
+      </c>
+      <c r="H372" s="4" t="s">
+        <v>2671</v>
+      </c>
+      <c r="I372" s="4" t="s">
+        <v>2455</v>
+      </c>
+      <c r="J372" s="4" t="s">
+        <v>2672</v>
+      </c>
+      <c r="K372" s="4" t="s">
+        <v>2673</v>
+      </c>
+      <c r="L372" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="M372" s="4" t="s">
+        <v>2674</v>
+      </c>
+    </row>
+    <row r="373" spans="1:13">
+      <c r="A373" s="4" t="s">
+        <v>2657</v>
+      </c>
+      <c r="B373" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C373" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D373" s="4" t="s">
+        <v>2675</v>
+      </c>
+      <c r="E373" s="4" t="s">
+        <v>2676</v>
+      </c>
+      <c r="F373" s="4" t="s">
+        <v>2677</v>
+      </c>
+      <c r="G373" s="4" t="s">
+        <v>2678</v>
+      </c>
+      <c r="H373" s="4" t="s">
+        <v>2679</v>
+      </c>
+      <c r="I373" s="4" t="s">
+        <v>2680</v>
+      </c>
+      <c r="J373" s="4" t="s">
+        <v>2681</v>
+      </c>
+      <c r="K373" s="4" t="s">
+        <v>2682</v>
+      </c>
+      <c r="L373" s="4" t="s">
+        <v>864</v>
+      </c>
+      <c r="M373" s="4" t="s">
+        <v>2683</v>
+      </c>
+    </row>
+    <row r="374" spans="1:13">
+      <c r="A374" s="4" t="s">
+        <v>2657</v>
+      </c>
+      <c r="B374" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C374" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D374" s="4" t="s">
+        <v>2684</v>
+      </c>
+      <c r="E374" s="4" t="s">
+        <v>2685</v>
+      </c>
+      <c r="F374" s="4" t="s">
+        <v>2686</v>
+      </c>
+      <c r="G374" s="4" t="s">
+        <v>2687</v>
+      </c>
+      <c r="H374" s="4" t="s">
+        <v>2688</v>
+      </c>
+      <c r="I374" s="4" t="s">
+        <v>2689</v>
+      </c>
+      <c r="J374" s="4" t="s">
+        <v>2690</v>
+      </c>
+      <c r="K374" s="4" t="s">
+        <v>2691</v>
+      </c>
+      <c r="L374" s="4" t="s">
+        <v>361</v>
+      </c>
+      <c r="M374" s="4" t="s">
+        <v>2692</v>
+      </c>
+    </row>
+    <row r="375" spans="1:13">
+      <c r="A375" s="4" t="s">
+        <v>2657</v>
+      </c>
+      <c r="B375" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C375" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D375" s="4" t="s">
+        <v>2693</v>
+      </c>
+      <c r="E375" s="4" t="s">
+        <v>2694</v>
+      </c>
+      <c r="F375" s="4" t="s">
+        <v>2695</v>
+      </c>
+      <c r="G375" s="4" t="s">
+        <v>2696</v>
+      </c>
+      <c r="H375" s="4" t="s">
+        <v>2697</v>
+      </c>
+      <c r="I375" s="4" t="s">
+        <v>2698</v>
+      </c>
+      <c r="J375" s="4" t="s">
+        <v>2699</v>
+      </c>
+      <c r="K375" s="4" t="s">
+        <v>2700</v>
+      </c>
+      <c r="L375" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="M375" s="4" t="s">
+        <v>2701</v>
+      </c>
+    </row>
+    <row r="376" spans="1:13">
+      <c r="A376" s="4" t="s">
+        <v>2657</v>
+      </c>
+      <c r="B376" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C376" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D376" s="4" t="s">
+        <v>2702</v>
+      </c>
+      <c r="E376" s="4" t="s">
+        <v>2703</v>
+      </c>
+      <c r="F376" s="4" t="s">
+        <v>2704</v>
+      </c>
+      <c r="G376" s="4" t="s">
+        <v>2705</v>
+      </c>
+      <c r="H376" s="4" t="s">
+        <v>2706</v>
+      </c>
+      <c r="I376" s="4" t="s">
+        <v>2707</v>
+      </c>
+      <c r="J376" s="4" t="s">
+        <v>2708</v>
+      </c>
+      <c r="K376" s="4" t="s">
+        <v>2709</v>
+      </c>
+      <c r="L376" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="M376" s="4" t="s">
+        <v>2710</v>
+      </c>
+    </row>
+    <row r="377" spans="1:13">
+      <c r="A377" s="4" t="s">
+        <v>2657</v>
+      </c>
+      <c r="B377" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C377" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D377" s="4" t="s">
+        <v>2711</v>
+      </c>
+      <c r="E377" s="4" t="s">
+        <v>2712</v>
+      </c>
+      <c r="F377" s="4" t="s">
+        <v>2713</v>
+      </c>
+      <c r="G377" s="4" t="s">
+        <v>2714</v>
+      </c>
+      <c r="H377" s="4" t="s">
+        <v>2715</v>
+      </c>
+      <c r="I377" s="4" t="s">
+        <v>2716</v>
+      </c>
+      <c r="J377" s="4" t="s">
+        <v>2717</v>
+      </c>
+      <c r="K377" s="4" t="s">
+        <v>2718</v>
+      </c>
+      <c r="L377" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="M377" s="4" t="s">
+        <v>2719</v>
+      </c>
+    </row>
+    <row r="378" spans="1:13">
+      <c r="A378" s="4" t="s">
+        <v>2720</v>
+      </c>
+      <c r="B378" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C378" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D378" s="4" t="s">
+        <v>2721</v>
+      </c>
+      <c r="E378" s="4" t="s">
+        <v>2722</v>
+      </c>
+      <c r="F378" s="4" t="s">
+        <v>2723</v>
+      </c>
+      <c r="G378" s="4" t="s">
+        <v>2724</v>
+      </c>
+      <c r="H378" s="4" t="s">
+        <v>2725</v>
+      </c>
+      <c r="I378" s="4" t="s">
+        <v>1941</v>
+      </c>
+      <c r="J378" s="4" t="s">
+        <v>2726</v>
+      </c>
+      <c r="K378" s="4" t="s">
+        <v>2727</v>
+      </c>
+      <c r="L378" s="4" t="s">
+        <v>536</v>
+      </c>
+      <c r="M378" s="4" t="s">
+        <v>2728</v>
+      </c>
+    </row>
+    <row r="379" spans="1:13">
+      <c r="A379" s="4" t="s">
+        <v>2720</v>
+      </c>
+      <c r="B379" s="4" t="s">
+        <v>2518</v>
+      </c>
+      <c r="C379" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D379" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="E379" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="F379" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="G379" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="H379" s="4" t="s">
+        <v>441</v>
+      </c>
+      <c r="I379" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J379" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="K379" s="4" t="s">
+        <v>629</v>
+      </c>
+      <c r="L379" s="4" t="s">
+        <v>2729</v>
+      </c>
+      <c r="M379" s="4" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="380" spans="1:13">
+      <c r="A380" s="4" t="s">
+        <v>2720</v>
+      </c>
+      <c r="B380" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C380" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D380" s="4" t="s">
+        <v>2730</v>
+      </c>
+      <c r="E380" s="4" t="s">
+        <v>2731</v>
+      </c>
+      <c r="F380" s="4" t="s">
+        <v>2732</v>
+      </c>
+      <c r="G380" s="4" t="s">
+        <v>2733</v>
+      </c>
+      <c r="H380" s="4" t="s">
+        <v>2734</v>
+      </c>
+      <c r="I380" s="4" t="s">
+        <v>2735</v>
+      </c>
+      <c r="J380" s="4" t="s">
+        <v>2736</v>
+      </c>
+      <c r="K380" s="4" t="s">
+        <v>2737</v>
+      </c>
+      <c r="L380" s="4" t="s">
+        <v>1683</v>
+      </c>
+      <c r="M380" s="4" t="s">
+        <v>2738</v>
+      </c>
+    </row>
+    <row r="381" spans="1:13">
+      <c r="A381" s="4" t="s">
+        <v>2720</v>
+      </c>
+      <c r="B381" s="4" t="s">
+        <v>2518</v>
+      </c>
+      <c r="C381" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D381" s="4" t="s">
+        <v>2739</v>
+      </c>
+      <c r="E381" s="4" t="s">
+        <v>2740</v>
+      </c>
+      <c r="F381" s="4" t="s">
+        <v>2741</v>
+      </c>
+      <c r="G381" s="4" t="s">
+        <v>2742</v>
+      </c>
+      <c r="H381" s="4" t="s">
+        <v>2743</v>
+      </c>
+      <c r="I381" s="4" t="s">
+        <v>1845</v>
+      </c>
+      <c r="J381" s="4" t="s">
+        <v>2744</v>
+      </c>
+      <c r="K381" s="4" t="s">
+        <v>2745</v>
+      </c>
+      <c r="L381" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="M381" s="4" t="s">
+        <v>2746</v>
+      </c>
+    </row>
+    <row r="382" spans="1:13">
+      <c r="A382" s="4" t="s">
+        <v>2720</v>
+      </c>
+      <c r="B382" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C382" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D382" s="4" t="s">
+        <v>2747</v>
+      </c>
+      <c r="E382" s="4" t="s">
+        <v>2748</v>
+      </c>
+      <c r="F382" s="4" t="s">
+        <v>2749</v>
+      </c>
+      <c r="G382" s="4" t="s">
+        <v>2750</v>
+      </c>
+      <c r="H382" s="4" t="s">
+        <v>2751</v>
+      </c>
+      <c r="I382" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="J382" s="4" t="s">
+        <v>2752</v>
+      </c>
+      <c r="K382" s="4" t="s">
+        <v>2753</v>
+      </c>
+      <c r="L382" s="4" t="s">
+        <v>992</v>
+      </c>
+      <c r="M382" s="4" t="s">
+        <v>2754</v>
+      </c>
+    </row>
+    <row r="383" spans="1:13">
+      <c r="A383" s="4" t="s">
+        <v>2720</v>
+      </c>
+      <c r="B383" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C383" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D383" s="4" t="s">
+        <v>2755</v>
+      </c>
+      <c r="E383" s="4" t="s">
+        <v>2756</v>
+      </c>
+      <c r="F383" s="4" t="s">
+        <v>2757</v>
+      </c>
+      <c r="G383" s="4" t="s">
+        <v>2758</v>
+      </c>
+      <c r="H383" s="4" t="s">
+        <v>2759</v>
+      </c>
+      <c r="I383" s="4" t="s">
+        <v>1810</v>
+      </c>
+      <c r="J383" s="4" t="s">
+        <v>2760</v>
+      </c>
+      <c r="K383" s="4" t="s">
+        <v>2761</v>
+      </c>
+      <c r="L383" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="M383" s="4" t="s">
+        <v>2762</v>
+      </c>
+    </row>
+    <row r="384" spans="1:13">
+      <c r="A384" s="4" t="s">
+        <v>2720</v>
+      </c>
+      <c r="B384" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C384" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D384" s="4" t="s">
+        <v>2763</v>
+      </c>
+      <c r="E384" s="4" t="s">
+        <v>2764</v>
+      </c>
+      <c r="F384" s="4" t="s">
+        <v>2765</v>
+      </c>
+      <c r="G384" s="4" t="s">
+        <v>2766</v>
+      </c>
+      <c r="H384" s="4" t="s">
+        <v>2767</v>
+      </c>
+      <c r="I384" s="4" t="s">
+        <v>2768</v>
+      </c>
+      <c r="J384" s="4" t="s">
+        <v>2769</v>
+      </c>
+      <c r="K384" s="4" t="s">
+        <v>2770</v>
+      </c>
+      <c r="L384" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="M384" s="4" t="s">
+        <v>2771</v>
+      </c>
+    </row>
+    <row r="385" spans="1:13">
+      <c r="A385" s="4" t="s">
+        <v>2720</v>
+      </c>
+      <c r="B385" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C385" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D385" s="4" t="s">
+        <v>2772</v>
+      </c>
+      <c r="E385" s="4" t="s">
+        <v>2773</v>
+      </c>
+      <c r="F385" s="4" t="s">
+        <v>2774</v>
+      </c>
+      <c r="G385" s="4" t="s">
+        <v>2775</v>
+      </c>
+      <c r="H385" s="4" t="s">
+        <v>2776</v>
+      </c>
+      <c r="I385" s="4" t="s">
+        <v>2777</v>
+      </c>
+      <c r="J385" s="4" t="s">
+        <v>2778</v>
+      </c>
+      <c r="K385" s="4" t="s">
+        <v>2779</v>
+      </c>
+      <c r="L385" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="M385" s="4" t="s">
+        <v>2780</v>
+      </c>
+    </row>
+    <row r="386" spans="1:13">
+      <c r="A386" s="4" t="s">
+        <v>2720</v>
+      </c>
+      <c r="B386" s="4" t="s">
+        <v>2518</v>
+      </c>
+      <c r="C386" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D386" s="4" t="s">
+        <v>2781</v>
+      </c>
+      <c r="E386" s="4" t="s">
+        <v>2782</v>
+      </c>
+      <c r="F386" s="4" t="s">
+        <v>2783</v>
+      </c>
+      <c r="G386" s="4" t="s">
+        <v>2784</v>
+      </c>
+      <c r="H386" s="4" t="s">
+        <v>1398</v>
+      </c>
+      <c r="I386" s="4" t="s">
+        <v>629</v>
+      </c>
+      <c r="J386" s="4" t="s">
+        <v>2785</v>
+      </c>
+      <c r="K386" s="4" t="s">
+        <v>2786</v>
+      </c>
+      <c r="L386" s="4" t="s">
+        <v>605</v>
+      </c>
+      <c r="M386" s="4" t="s">
+        <v>2787</v>
+      </c>
+    </row>
+    <row r="387" spans="1:13">
+      <c r="A387" s="4" t="s">
+        <v>2720</v>
+      </c>
+      <c r="B387" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C387" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D387" s="4" t="s">
+        <v>2788</v>
+      </c>
+      <c r="E387" s="4" t="s">
+        <v>2789</v>
+      </c>
+      <c r="F387" s="4" t="s">
+        <v>2790</v>
+      </c>
+      <c r="G387" s="4" t="s">
+        <v>2791</v>
+      </c>
+      <c r="H387" s="4" t="s">
+        <v>2792</v>
+      </c>
+      <c r="I387" s="4" t="s">
+        <v>953</v>
+      </c>
+      <c r="J387" s="4" t="s">
+        <v>2793</v>
+      </c>
+      <c r="K387" s="4" t="s">
+        <v>2794</v>
+      </c>
+      <c r="L387" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="M387" s="4" t="s">
+        <v>2795</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:Z333" etc:filterBottomFollowUsedRange="0">
+  <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:Z352" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="0">
-      <filters>
-        <filter val="2026-08-07"/>
-      </filters>
+      <customFilters>
+        <customFilter operator="equal" val="2026-08-07"/>
+      </customFilters>
     </filterColumn>
     <filterColumn colId="1">
-      <filters>
-        <filter val="爆量算法池"/>
-        <filter val="大神"/>
-      </filters>
+      <customFilters>
+        <customFilter operator="equal" val="爆量算法池"/>
+        <customFilter operator="equal" val="大神"/>
+      </customFilters>
     </filterColumn>
-    <sortState ref="A2:Z333">
+    <sortState ref="A1:Z352">
       <sortCondition ref="B1"/>
     </sortState>
     <extLst/>

</xml_diff>

<commit_message>
feat: add daily broadcast panel
</commit_message>
<xml_diff>
--- a/data/uploads/tongshi_demo.xlsx
+++ b/data/uploads/tongshi_demo.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28000" windowHeight="11140"/>
+    <workbookView windowWidth="26860" windowHeight="11140"/>
   </bookViews>
   <sheets>
     <sheet name="sheet" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4576" uniqueCount="2788">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4687" uniqueCount="2792">
   <si>
     <t>日期</t>
   </si>
@@ -8394,6 +8394,18 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>20260821</t>
+  </si>
+  <si>
+    <t>20260822</t>
+  </si>
+  <si>
+    <t>20260823</t>
+  </si>
+  <si>
+    <t>20260824</t>
   </si>
 </sst>
 </file>
@@ -9427,7 +9439,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:Z435"/>
+  <dimension ref="A1:Z471"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="16.0192307692308" style="2" customWidth="1"/>
@@ -27259,6 +27271,1482 @@
         <v>1</v>
       </c>
     </row>
+    <row r="436" s="1" customFormat="1" spans="1:13">
+      <c r="A436" s="1" t="s">
+        <v>2788</v>
+      </c>
+      <c r="B436" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C436" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D436" s="1">
+        <v>0.00313070265021513</v>
+      </c>
+      <c r="E436" s="1">
+        <v>341757</v>
+      </c>
+      <c r="F436" s="1">
+        <v>59731</v>
+      </c>
+      <c r="G436" s="1">
+        <v>12399</v>
+      </c>
+      <c r="H436" s="1">
+        <v>8858</v>
+      </c>
+      <c r="I436" s="1">
+        <v>187</v>
+      </c>
+      <c r="J436" s="1">
+        <v>1491706</v>
+      </c>
+      <c r="K436" s="1">
+        <v>664214</v>
+      </c>
+      <c r="L436" s="1">
+        <v>0.892832755329731</v>
+      </c>
+      <c r="M436" s="1">
+        <v>69087</v>
+      </c>
+    </row>
+    <row r="437" s="1" customFormat="1" spans="1:13">
+      <c r="A437" s="1" t="s">
+        <v>2788</v>
+      </c>
+      <c r="B437" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C437" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D437" s="1">
+        <v>0.00313070265021513</v>
+      </c>
+      <c r="E437" s="1">
+        <v>341757</v>
+      </c>
+      <c r="F437" s="1">
+        <v>59731</v>
+      </c>
+      <c r="G437" s="1">
+        <v>12399</v>
+      </c>
+      <c r="H437" s="1">
+        <v>8858</v>
+      </c>
+      <c r="I437" s="1">
+        <v>187</v>
+      </c>
+      <c r="J437" s="1">
+        <v>1491706</v>
+      </c>
+      <c r="K437" s="1">
+        <v>664214</v>
+      </c>
+      <c r="L437" s="1">
+        <v>0.892832755329731</v>
+      </c>
+      <c r="M437" s="1">
+        <v>69087</v>
+      </c>
+    </row>
+    <row r="438" s="1" customFormat="1" spans="1:13">
+      <c r="A438" s="1" t="s">
+        <v>2788</v>
+      </c>
+      <c r="B438" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C438" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D438" s="1">
+        <v>0.000714616810877627</v>
+      </c>
+      <c r="E438" s="1">
+        <v>268190</v>
+      </c>
+      <c r="F438" s="1">
+        <v>51776</v>
+      </c>
+      <c r="G438" s="1">
+        <v>4257</v>
+      </c>
+      <c r="H438" s="1">
+        <v>3503</v>
+      </c>
+      <c r="I438" s="1">
+        <v>37</v>
+      </c>
+      <c r="J438" s="1">
+        <v>1083836</v>
+      </c>
+      <c r="K438" s="1">
+        <v>279802</v>
+      </c>
+      <c r="L438" s="1">
+        <v>1.09545846057474</v>
+      </c>
+      <c r="M438" s="1">
+        <v>56653</v>
+      </c>
+    </row>
+    <row r="439" s="1" customFormat="1" spans="1:13">
+      <c r="A439" s="1" t="s">
+        <v>2788</v>
+      </c>
+      <c r="B439" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C439" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D439" s="1">
+        <v>0.00444972956384978</v>
+      </c>
+      <c r="E439" s="1">
+        <v>206379</v>
+      </c>
+      <c r="F439" s="1">
+        <v>26069</v>
+      </c>
+      <c r="G439" s="1">
+        <v>5741</v>
+      </c>
+      <c r="H439" s="1">
+        <v>4023</v>
+      </c>
+      <c r="I439" s="1">
+        <v>116</v>
+      </c>
+      <c r="J439" s="1">
+        <v>686673</v>
+      </c>
+      <c r="K439" s="1">
+        <v>352068</v>
+      </c>
+      <c r="L439" s="1">
+        <v>1.0220867444696</v>
+      </c>
+      <c r="M439" s="1">
+        <v>31085</v>
+      </c>
+    </row>
+    <row r="440" s="1" customFormat="1" spans="1:13">
+      <c r="A440" s="1" t="s">
+        <v>2788</v>
+      </c>
+      <c r="B440" s="1" t="s">
+        <v>2658</v>
+      </c>
+      <c r="C440" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D440" s="1">
+        <v>0.00434038778355088</v>
+      </c>
+      <c r="E440" s="1">
+        <v>262977</v>
+      </c>
+      <c r="F440" s="1">
+        <v>63128</v>
+      </c>
+      <c r="G440" s="1">
+        <v>19346</v>
+      </c>
+      <c r="H440" s="1">
+        <v>11699</v>
+      </c>
+      <c r="I440" s="1">
+        <v>274</v>
+      </c>
+      <c r="J440" s="1">
+        <v>1321752</v>
+      </c>
+      <c r="K440" s="1">
+        <v>570320</v>
+      </c>
+      <c r="L440" s="1">
+        <v>0.491333264412971</v>
+      </c>
+      <c r="M440" s="1">
+        <v>69789</v>
+      </c>
+    </row>
+    <row r="441" s="1" customFormat="1" spans="1:13">
+      <c r="A441" s="1" t="s">
+        <v>2788</v>
+      </c>
+      <c r="B441" s="1" t="s">
+        <v>2661</v>
+      </c>
+      <c r="C441" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D441" s="1">
+        <v>0.010272759475735</v>
+      </c>
+      <c r="E441" s="1">
+        <v>7647</v>
+      </c>
+      <c r="F441" s="1">
+        <v>2823</v>
+      </c>
+      <c r="G441" s="1">
+        <v>1434</v>
+      </c>
+      <c r="H441" s="1">
+        <v>1203</v>
+      </c>
+      <c r="I441" s="1">
+        <v>29</v>
+      </c>
+      <c r="J441" s="1">
+        <v>71849</v>
+      </c>
+      <c r="K441" s="1">
+        <v>42992</v>
+      </c>
+      <c r="L441" s="1">
+        <v>0.499674569967457</v>
+      </c>
+      <c r="M441" s="1">
+        <v>3256</v>
+      </c>
+    </row>
+    <row r="442" s="1" customFormat="1" spans="1:13">
+      <c r="A442" s="1" t="s">
+        <v>2788</v>
+      </c>
+      <c r="B442" s="1" t="s">
+        <v>2661</v>
+      </c>
+      <c r="C442" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D442" s="1">
+        <v>0.0178260869565217</v>
+      </c>
+      <c r="E442" s="1">
+        <v>7193</v>
+      </c>
+      <c r="F442" s="1">
+        <v>2300</v>
+      </c>
+      <c r="G442" s="1">
+        <v>1309</v>
+      </c>
+      <c r="H442" s="1">
+        <v>1094</v>
+      </c>
+      <c r="I442" s="1">
+        <v>41</v>
+      </c>
+      <c r="J442" s="1">
+        <v>74822</v>
+      </c>
+      <c r="K442" s="1">
+        <v>52666</v>
+      </c>
+      <c r="L442" s="1">
+        <v>0.670562770562771</v>
+      </c>
+      <c r="M442" s="1">
+        <v>2911</v>
+      </c>
+    </row>
+    <row r="443" s="1" customFormat="1" spans="1:13">
+      <c r="A443" s="1" t="s">
+        <v>2788</v>
+      </c>
+      <c r="B443" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C443" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D443" s="1">
+        <v>0.00777352716143841</v>
+      </c>
+      <c r="E443" s="1">
+        <v>228242</v>
+      </c>
+      <c r="F443" s="1">
+        <v>32675</v>
+      </c>
+      <c r="G443" s="1">
+        <v>10316</v>
+      </c>
+      <c r="H443" s="1">
+        <v>7245</v>
+      </c>
+      <c r="I443" s="1">
+        <v>254</v>
+      </c>
+      <c r="J443" s="1">
+        <v>1158348</v>
+      </c>
+      <c r="K443" s="1">
+        <v>750566</v>
+      </c>
+      <c r="L443" s="1">
+        <v>1.21262440222308</v>
+      </c>
+      <c r="M443" s="1">
+        <v>43463</v>
+      </c>
+    </row>
+    <row r="444" s="1" customFormat="1" spans="1:13">
+      <c r="A444" s="1" t="s">
+        <v>2788</v>
+      </c>
+      <c r="B444" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C444" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D444" s="1">
+        <v>0.00124432629629106</v>
+      </c>
+      <c r="E444" s="1">
+        <v>261129</v>
+      </c>
+      <c r="F444" s="1">
+        <v>70721</v>
+      </c>
+      <c r="G444" s="1">
+        <v>6991</v>
+      </c>
+      <c r="H444" s="1">
+        <v>5647</v>
+      </c>
+      <c r="I444" s="1">
+        <v>88</v>
+      </c>
+      <c r="J444" s="1">
+        <v>1600046</v>
+      </c>
+      <c r="K444" s="1">
+        <v>490559</v>
+      </c>
+      <c r="L444" s="1">
+        <v>1.1695012635293</v>
+      </c>
+      <c r="M444" s="1">
+        <v>79003</v>
+      </c>
+    </row>
+    <row r="445" s="1" customFormat="1" spans="1:13">
+      <c r="A445" s="1" t="s">
+        <v>2788</v>
+      </c>
+      <c r="B445" s="1" t="s">
+        <v>2658</v>
+      </c>
+      <c r="C445" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D445" s="1">
+        <v>0.00882744237891482</v>
+      </c>
+      <c r="E445" s="1">
+        <v>237659</v>
+      </c>
+      <c r="F445" s="1">
+        <v>55622</v>
+      </c>
+      <c r="G445" s="1">
+        <v>17963</v>
+      </c>
+      <c r="H445" s="1">
+        <v>10958</v>
+      </c>
+      <c r="I445" s="1">
+        <v>491</v>
+      </c>
+      <c r="J445" s="1">
+        <v>1382296</v>
+      </c>
+      <c r="K445" s="1">
+        <v>707907</v>
+      </c>
+      <c r="L445" s="1">
+        <v>0.656819573567889</v>
+      </c>
+      <c r="M445" s="1">
+        <v>64858</v>
+      </c>
+    </row>
+    <row r="446" spans="1:13">
+      <c r="A446" s="1" t="s">
+        <v>2789</v>
+      </c>
+      <c r="B446" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C446" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D446" s="1">
+        <v>0.00230777552075195</v>
+      </c>
+      <c r="E446" s="1">
+        <v>446369</v>
+      </c>
+      <c r="F446" s="1">
+        <v>83197</v>
+      </c>
+      <c r="G446" s="1">
+        <v>16727</v>
+      </c>
+      <c r="H446" s="1">
+        <v>11492</v>
+      </c>
+      <c r="I446" s="1">
+        <v>192</v>
+      </c>
+      <c r="J446" s="1">
+        <v>1954156</v>
+      </c>
+      <c r="K446" s="1">
+        <v>795743</v>
+      </c>
+      <c r="L446" s="1">
+        <v>0.792872800462326</v>
+      </c>
+      <c r="M446" s="1">
+        <v>94442</v>
+      </c>
+    </row>
+    <row r="447" spans="1:13">
+      <c r="A447" s="1" t="s">
+        <v>2789</v>
+      </c>
+      <c r="B447" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C447" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D447" s="1">
+        <v>0.00286060072615249</v>
+      </c>
+      <c r="E447" s="1">
+        <v>206536</v>
+      </c>
+      <c r="F447" s="1">
+        <v>27267</v>
+      </c>
+      <c r="G447" s="1">
+        <v>5954</v>
+      </c>
+      <c r="H447" s="1">
+        <v>4079</v>
+      </c>
+      <c r="I447" s="1">
+        <v>78</v>
+      </c>
+      <c r="J447" s="1">
+        <v>661690</v>
+      </c>
+      <c r="K447" s="1">
+        <v>306033</v>
+      </c>
+      <c r="L447" s="1">
+        <v>0.856659388646288</v>
+      </c>
+      <c r="M447" s="1">
+        <v>31537</v>
+      </c>
+    </row>
+    <row r="448" spans="1:13">
+      <c r="A448" s="1" t="s">
+        <v>2789</v>
+      </c>
+      <c r="B448" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C448" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D448" s="1">
+        <v>0.000635011350827896</v>
+      </c>
+      <c r="E448" s="1">
+        <v>354254</v>
+      </c>
+      <c r="F448" s="1">
+        <v>62991</v>
+      </c>
+      <c r="G448" s="1">
+        <v>5488</v>
+      </c>
+      <c r="H448" s="1">
+        <v>4497</v>
+      </c>
+      <c r="I448" s="1">
+        <v>40</v>
+      </c>
+      <c r="J448" s="1">
+        <v>1358353</v>
+      </c>
+      <c r="K448" s="1">
+        <v>349445</v>
+      </c>
+      <c r="L448" s="1">
+        <v>1.0612396744412</v>
+      </c>
+      <c r="M448" s="1">
+        <v>69146</v>
+      </c>
+    </row>
+    <row r="449" spans="1:13">
+      <c r="A449" s="1" t="s">
+        <v>2789</v>
+      </c>
+      <c r="B449" s="1" t="s">
+        <v>2658</v>
+      </c>
+      <c r="C449" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D449" s="1">
+        <v>0.00449846446645616</v>
+      </c>
+      <c r="E449" s="1">
+        <v>174319</v>
+      </c>
+      <c r="F449" s="1">
+        <v>46238</v>
+      </c>
+      <c r="G449" s="1">
+        <v>18076</v>
+      </c>
+      <c r="H449" s="1">
+        <v>10119</v>
+      </c>
+      <c r="I449" s="1">
+        <v>208</v>
+      </c>
+      <c r="J449" s="1">
+        <v>989774</v>
+      </c>
+      <c r="K449" s="1">
+        <v>469460</v>
+      </c>
+      <c r="L449" s="1">
+        <v>0.432857564357896</v>
+      </c>
+      <c r="M449" s="1">
+        <v>51580</v>
+      </c>
+    </row>
+    <row r="450" spans="1:13">
+      <c r="A450" s="1" t="s">
+        <v>2789</v>
+      </c>
+      <c r="B450" s="1" t="s">
+        <v>2661</v>
+      </c>
+      <c r="C450" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D450" s="1">
+        <v>0.00966486757876239</v>
+      </c>
+      <c r="E450" s="1">
+        <v>20042</v>
+      </c>
+      <c r="F450" s="1">
+        <v>7967</v>
+      </c>
+      <c r="G450" s="1">
+        <v>4063</v>
+      </c>
+      <c r="H450" s="1">
+        <v>3457</v>
+      </c>
+      <c r="I450" s="1">
+        <v>77</v>
+      </c>
+      <c r="J450" s="1">
+        <v>214244</v>
+      </c>
+      <c r="K450" s="1">
+        <v>134993</v>
+      </c>
+      <c r="L450" s="1">
+        <v>0.553749282139634</v>
+      </c>
+      <c r="M450" s="1">
+        <v>9435</v>
+      </c>
+    </row>
+    <row r="451" spans="1:13">
+      <c r="A451" s="1" t="s">
+        <v>2789</v>
+      </c>
+      <c r="B451" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C451" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D451" s="1">
+        <v>0.000927500386458494</v>
+      </c>
+      <c r="E451" s="1">
+        <v>206867</v>
+      </c>
+      <c r="F451" s="1">
+        <v>51752</v>
+      </c>
+      <c r="G451" s="1">
+        <v>6034</v>
+      </c>
+      <c r="H451" s="1">
+        <v>4766</v>
+      </c>
+      <c r="I451" s="1">
+        <v>48</v>
+      </c>
+      <c r="J451" s="1">
+        <v>1145521</v>
+      </c>
+      <c r="K451" s="1">
+        <v>328299</v>
+      </c>
+      <c r="L451" s="1">
+        <v>0.906803115677826</v>
+      </c>
+      <c r="M451" s="1">
+        <v>57137</v>
+      </c>
+    </row>
+    <row r="452" spans="1:13">
+      <c r="A452" s="1" t="s">
+        <v>2789</v>
+      </c>
+      <c r="B452" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C452" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D452" s="1">
+        <v>0.00419054777788218</v>
+      </c>
+      <c r="E452" s="1">
+        <v>397059</v>
+      </c>
+      <c r="F452" s="1">
+        <v>53215</v>
+      </c>
+      <c r="G452" s="1">
+        <v>10646</v>
+      </c>
+      <c r="H452" s="1">
+        <v>7701</v>
+      </c>
+      <c r="I452" s="1">
+        <v>223</v>
+      </c>
+      <c r="J452" s="1">
+        <v>1443735</v>
+      </c>
+      <c r="K452" s="1">
+        <v>700444</v>
+      </c>
+      <c r="L452" s="1">
+        <v>1.09656835118041</v>
+      </c>
+      <c r="M452" s="1">
+        <v>63732</v>
+      </c>
+    </row>
+    <row r="453" spans="1:13">
+      <c r="A453" s="1" t="s">
+        <v>2789</v>
+      </c>
+      <c r="B453" s="1" t="s">
+        <v>2658</v>
+      </c>
+      <c r="C453" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D453" s="1">
+        <v>0.00831980179788071</v>
+      </c>
+      <c r="E453" s="1">
+        <v>277788</v>
+      </c>
+      <c r="F453" s="1">
+        <v>59737</v>
+      </c>
+      <c r="G453" s="1">
+        <v>18292</v>
+      </c>
+      <c r="H453" s="1">
+        <v>11012</v>
+      </c>
+      <c r="I453" s="1">
+        <v>497</v>
+      </c>
+      <c r="J453" s="1">
+        <v>1418397</v>
+      </c>
+      <c r="K453" s="1">
+        <v>689174</v>
+      </c>
+      <c r="L453" s="1">
+        <v>0.62793753189008</v>
+      </c>
+      <c r="M453" s="1">
+        <v>68771</v>
+      </c>
+    </row>
+    <row r="454" spans="1:13">
+      <c r="A454" s="1" t="s">
+        <v>2789</v>
+      </c>
+      <c r="B454" s="1" t="s">
+        <v>2661</v>
+      </c>
+      <c r="C454" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D454" s="1">
+        <v>0.0185471406491499</v>
+      </c>
+      <c r="E454" s="1">
+        <v>2307</v>
+      </c>
+      <c r="F454" s="1">
+        <v>647</v>
+      </c>
+      <c r="G454" s="1">
+        <v>402</v>
+      </c>
+      <c r="H454" s="1">
+        <v>343</v>
+      </c>
+      <c r="I454" s="1">
+        <v>12</v>
+      </c>
+      <c r="J454" s="1">
+        <v>22330</v>
+      </c>
+      <c r="K454" s="1">
+        <v>17057</v>
+      </c>
+      <c r="L454" s="1">
+        <v>0.707172470978441</v>
+      </c>
+      <c r="M454" s="1">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="455" spans="1:13">
+      <c r="A455" s="1" t="s">
+        <v>2790</v>
+      </c>
+      <c r="B455" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C455" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D455" s="1">
+        <v>0.00133877769596359</v>
+      </c>
+      <c r="E455" s="1">
+        <v>516796</v>
+      </c>
+      <c r="F455" s="1">
+        <v>89634</v>
+      </c>
+      <c r="G455" s="1">
+        <v>16150</v>
+      </c>
+      <c r="H455" s="1">
+        <v>11166</v>
+      </c>
+      <c r="I455" s="1">
+        <v>120</v>
+      </c>
+      <c r="J455" s="1">
+        <v>1935602</v>
+      </c>
+      <c r="K455" s="1">
+        <v>662681</v>
+      </c>
+      <c r="L455" s="1">
+        <v>0.683881320949432</v>
+      </c>
+      <c r="M455" s="1">
+        <v>98915</v>
+      </c>
+    </row>
+    <row r="456" spans="1:13">
+      <c r="A456" s="1" t="s">
+        <v>2790</v>
+      </c>
+      <c r="B456" s="1" t="s">
+        <v>2658</v>
+      </c>
+      <c r="C456" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D456" s="1">
+        <v>0.00311826919985855</v>
+      </c>
+      <c r="E456" s="1">
+        <v>251608</v>
+      </c>
+      <c r="F456" s="1">
+        <v>62214</v>
+      </c>
+      <c r="G456" s="1">
+        <v>12520</v>
+      </c>
+      <c r="H456" s="1">
+        <v>8045</v>
+      </c>
+      <c r="I456" s="1">
+        <v>194</v>
+      </c>
+      <c r="J456" s="1">
+        <v>1267322</v>
+      </c>
+      <c r="K456" s="1">
+        <v>432037</v>
+      </c>
+      <c r="L456" s="1">
+        <v>0.575129126730564</v>
+      </c>
+      <c r="M456" s="1">
+        <v>68019</v>
+      </c>
+    </row>
+    <row r="457" spans="1:13">
+      <c r="A457" s="1" t="s">
+        <v>2790</v>
+      </c>
+      <c r="B457" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C457" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D457" s="1">
+        <v>0.000622719110235764</v>
+      </c>
+      <c r="E457" s="1">
+        <v>390014</v>
+      </c>
+      <c r="F457" s="1">
+        <v>69052</v>
+      </c>
+      <c r="G457" s="1">
+        <v>4582</v>
+      </c>
+      <c r="H457" s="1">
+        <v>3836</v>
+      </c>
+      <c r="I457" s="1">
+        <v>43</v>
+      </c>
+      <c r="J457" s="1">
+        <v>1399666</v>
+      </c>
+      <c r="K457" s="1">
+        <v>298512</v>
+      </c>
+      <c r="L457" s="1">
+        <v>1.08581405499782</v>
+      </c>
+      <c r="M457" s="1">
+        <v>74756</v>
+      </c>
+    </row>
+    <row r="458" spans="1:13">
+      <c r="A458" s="1" t="s">
+        <v>2790</v>
+      </c>
+      <c r="B458" s="1" t="s">
+        <v>2661</v>
+      </c>
+      <c r="C458" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D458" s="1">
+        <v>0.0097058384351202</v>
+      </c>
+      <c r="E458" s="1">
+        <v>19765</v>
+      </c>
+      <c r="F458" s="1">
+        <v>6697</v>
+      </c>
+      <c r="G458" s="1">
+        <v>3265</v>
+      </c>
+      <c r="H458" s="1">
+        <v>2796</v>
+      </c>
+      <c r="I458" s="1">
+        <v>65</v>
+      </c>
+      <c r="J458" s="1">
+        <v>177062</v>
+      </c>
+      <c r="K458" s="1">
+        <v>110380</v>
+      </c>
+      <c r="L458" s="1">
+        <v>0.563450740173558</v>
+      </c>
+      <c r="M458" s="1">
+        <v>7912</v>
+      </c>
+    </row>
+    <row r="459" spans="1:13">
+      <c r="A459" s="1" t="s">
+        <v>2790</v>
+      </c>
+      <c r="B459" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C459" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D459" s="1">
+        <v>0.00286630392537894</v>
+      </c>
+      <c r="E459" s="1">
+        <v>210179</v>
+      </c>
+      <c r="F459" s="1">
+        <v>20584</v>
+      </c>
+      <c r="G459" s="1">
+        <v>4220</v>
+      </c>
+      <c r="H459" s="1">
+        <v>2918</v>
+      </c>
+      <c r="I459" s="1">
+        <v>59</v>
+      </c>
+      <c r="J459" s="1">
+        <v>497278</v>
+      </c>
+      <c r="K459" s="1">
+        <v>220111</v>
+      </c>
+      <c r="L459" s="1">
+        <v>0.869316745655608</v>
+      </c>
+      <c r="M459" s="1">
+        <v>23725</v>
+      </c>
+    </row>
+    <row r="460" spans="1:13">
+      <c r="A460" s="1" t="s">
+        <v>2790</v>
+      </c>
+      <c r="B460" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C460" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D460" s="1">
+        <v>0.000423539901917075</v>
+      </c>
+      <c r="E460" s="1">
+        <v>306936</v>
+      </c>
+      <c r="F460" s="1">
+        <v>89720</v>
+      </c>
+      <c r="G460" s="1">
+        <v>6628</v>
+      </c>
+      <c r="H460" s="1">
+        <v>5378</v>
+      </c>
+      <c r="I460" s="1">
+        <v>38</v>
+      </c>
+      <c r="J460" s="1">
+        <v>1823506</v>
+      </c>
+      <c r="K460" s="1">
+        <v>369903</v>
+      </c>
+      <c r="L460" s="1">
+        <v>0.930152383826192</v>
+      </c>
+      <c r="M460" s="1">
+        <v>96636</v>
+      </c>
+    </row>
+    <row r="461" spans="1:13">
+      <c r="A461" s="1" t="s">
+        <v>2790</v>
+      </c>
+      <c r="B461" s="1" t="s">
+        <v>2661</v>
+      </c>
+      <c r="C461" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D461" s="1">
+        <v>0.0234375</v>
+      </c>
+      <c r="E461" s="1">
+        <v>1017</v>
+      </c>
+      <c r="F461" s="1">
+        <v>128</v>
+      </c>
+      <c r="G461" s="1">
+        <v>77</v>
+      </c>
+      <c r="H461" s="1">
+        <v>66</v>
+      </c>
+      <c r="I461" s="1">
+        <v>3</v>
+      </c>
+      <c r="J461" s="1">
+        <v>4088</v>
+      </c>
+      <c r="K461" s="1">
+        <v>2901</v>
+      </c>
+      <c r="L461" s="1">
+        <v>0.627922077922078</v>
+      </c>
+      <c r="M461" s="1">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="462" spans="1:13">
+      <c r="A462" s="1" t="s">
+        <v>2790</v>
+      </c>
+      <c r="B462" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C462" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D462" s="1">
+        <v>0.00264300306435138</v>
+      </c>
+      <c r="E462" s="1">
+        <v>615040</v>
+      </c>
+      <c r="F462" s="1">
+        <v>78320</v>
+      </c>
+      <c r="G462" s="1">
+        <v>12387</v>
+      </c>
+      <c r="H462" s="1">
+        <v>9340</v>
+      </c>
+      <c r="I462" s="1">
+        <v>207</v>
+      </c>
+      <c r="J462" s="1">
+        <v>1930335</v>
+      </c>
+      <c r="K462" s="1">
+        <v>799513</v>
+      </c>
+      <c r="L462" s="1">
+        <v>1.07574204138748</v>
+      </c>
+      <c r="M462" s="1">
+        <v>90662</v>
+      </c>
+    </row>
+    <row r="463" spans="1:13">
+      <c r="A463" s="1" t="s">
+        <v>2790</v>
+      </c>
+      <c r="B463" s="1" t="s">
+        <v>2658</v>
+      </c>
+      <c r="C463" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D463" s="1">
+        <v>0.0035233483861363</v>
+      </c>
+      <c r="E463" s="1">
+        <v>511868</v>
+      </c>
+      <c r="F463" s="1">
+        <v>141059</v>
+      </c>
+      <c r="G463" s="1">
+        <v>21950</v>
+      </c>
+      <c r="H463" s="1">
+        <v>14749</v>
+      </c>
+      <c r="I463" s="1">
+        <v>497</v>
+      </c>
+      <c r="J463" s="1">
+        <v>2816202</v>
+      </c>
+      <c r="K463" s="1">
+        <v>903087</v>
+      </c>
+      <c r="L463" s="1">
+        <v>0.685715261958998</v>
+      </c>
+      <c r="M463" s="1">
+        <v>154108</v>
+      </c>
+    </row>
+    <row r="464" spans="1:13">
+      <c r="A464" s="1" t="s">
+        <v>2791</v>
+      </c>
+      <c r="B464" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C464" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D464" s="1">
+        <v>0</v>
+      </c>
+      <c r="E464" s="1">
+        <v>19</v>
+      </c>
+      <c r="F464" s="1">
+        <v>5</v>
+      </c>
+      <c r="G464" s="1">
+        <v>0</v>
+      </c>
+      <c r="H464" s="1">
+        <v>0</v>
+      </c>
+      <c r="I464" s="1">
+        <v>0</v>
+      </c>
+      <c r="J464" s="1">
+        <v>64</v>
+      </c>
+      <c r="K464" s="1">
+        <v>0</v>
+      </c>
+      <c r="L464" s="1" t="s">
+        <v>2787</v>
+      </c>
+      <c r="M464" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="465" spans="1:13">
+      <c r="A465" s="1" t="s">
+        <v>2791</v>
+      </c>
+      <c r="B465" s="1" t="s">
+        <v>2661</v>
+      </c>
+      <c r="C465" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D465" s="1" t="s">
+        <v>2787</v>
+      </c>
+      <c r="E465" s="1">
+        <v>1</v>
+      </c>
+      <c r="F465" s="1">
+        <v>0</v>
+      </c>
+      <c r="G465" s="1">
+        <v>0</v>
+      </c>
+      <c r="H465" s="1">
+        <v>0</v>
+      </c>
+      <c r="I465" s="1">
+        <v>0</v>
+      </c>
+      <c r="J465" s="1">
+        <v>0</v>
+      </c>
+      <c r="K465" s="1">
+        <v>0</v>
+      </c>
+      <c r="L465" s="1" t="s">
+        <v>2787</v>
+      </c>
+      <c r="M465" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="466" spans="1:13">
+      <c r="A466" s="1" t="s">
+        <v>2791</v>
+      </c>
+      <c r="B466" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C466" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D466" s="1">
+        <v>0</v>
+      </c>
+      <c r="E466" s="1">
+        <v>19</v>
+      </c>
+      <c r="F466" s="1">
+        <v>3</v>
+      </c>
+      <c r="G466" s="1">
+        <v>1</v>
+      </c>
+      <c r="H466" s="1">
+        <v>1</v>
+      </c>
+      <c r="I466" s="1">
+        <v>0</v>
+      </c>
+      <c r="J466" s="1">
+        <v>72</v>
+      </c>
+      <c r="K466" s="1">
+        <v>12</v>
+      </c>
+      <c r="L466" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="M466" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="467" spans="1:13">
+      <c r="A467" s="1" t="s">
+        <v>2791</v>
+      </c>
+      <c r="B467" s="1" t="s">
+        <v>2658</v>
+      </c>
+      <c r="C467" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D467" s="1">
+        <v>0.00410576449334866</v>
+      </c>
+      <c r="E467" s="1">
+        <v>51444</v>
+      </c>
+      <c r="F467" s="1">
+        <v>18267</v>
+      </c>
+      <c r="G467" s="1">
+        <v>3584</v>
+      </c>
+      <c r="H467" s="1">
+        <v>2170</v>
+      </c>
+      <c r="I467" s="1">
+        <v>75</v>
+      </c>
+      <c r="J467" s="1">
+        <v>372861</v>
+      </c>
+      <c r="K467" s="1">
+        <v>117798</v>
+      </c>
+      <c r="L467" s="1">
+        <v>0.547795758928571</v>
+      </c>
+      <c r="M467" s="1">
+        <v>19920</v>
+      </c>
+    </row>
+    <row r="468" spans="1:13">
+      <c r="A468" s="1" t="s">
+        <v>2791</v>
+      </c>
+      <c r="B468" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C468" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D468" s="1">
+        <v>0.000926406284740236</v>
+      </c>
+      <c r="E468" s="1">
+        <v>236872</v>
+      </c>
+      <c r="F468" s="1">
+        <v>53972</v>
+      </c>
+      <c r="G468" s="1">
+        <v>4319</v>
+      </c>
+      <c r="H468" s="1">
+        <v>3483</v>
+      </c>
+      <c r="I468" s="1">
+        <v>50</v>
+      </c>
+      <c r="J468" s="1">
+        <v>1075151</v>
+      </c>
+      <c r="K468" s="1">
+        <v>275551</v>
+      </c>
+      <c r="L468" s="1">
+        <v>1.06332870263178</v>
+      </c>
+      <c r="M468" s="1">
+        <v>58612</v>
+      </c>
+    </row>
+    <row r="469" spans="1:13">
+      <c r="A469" s="1" t="s">
+        <v>2791</v>
+      </c>
+      <c r="B469" s="1" t="s">
+        <v>2658</v>
+      </c>
+      <c r="C469" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D469" s="1">
+        <v>0.0104905223556649</v>
+      </c>
+      <c r="E469" s="1">
+        <v>71095</v>
+      </c>
+      <c r="F469" s="1">
+        <v>13822</v>
+      </c>
+      <c r="G469" s="1">
+        <v>3367</v>
+      </c>
+      <c r="H469" s="1">
+        <v>2105</v>
+      </c>
+      <c r="I469" s="1">
+        <v>145</v>
+      </c>
+      <c r="J469" s="1">
+        <v>337725</v>
+      </c>
+      <c r="K469" s="1">
+        <v>153451</v>
+      </c>
+      <c r="L469" s="1">
+        <v>0.75958320958321</v>
+      </c>
+      <c r="M469" s="1">
+        <v>16029</v>
+      </c>
+    </row>
+    <row r="470" spans="1:13">
+      <c r="A470" s="1" t="s">
+        <v>2791</v>
+      </c>
+      <c r="B470" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C470" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D470" s="1">
+        <v>0.00124494242141301</v>
+      </c>
+      <c r="E470" s="1">
+        <v>122252</v>
+      </c>
+      <c r="F470" s="1">
+        <v>25704</v>
+      </c>
+      <c r="G470" s="1">
+        <v>3073</v>
+      </c>
+      <c r="H470" s="1">
+        <v>2376</v>
+      </c>
+      <c r="I470" s="1">
+        <v>32</v>
+      </c>
+      <c r="J470" s="1">
+        <v>581149</v>
+      </c>
+      <c r="K470" s="1">
+        <v>198591</v>
+      </c>
+      <c r="L470" s="1">
+        <v>1.07707452001302</v>
+      </c>
+      <c r="M470" s="1">
+        <v>28829</v>
+      </c>
+    </row>
+    <row r="471" spans="1:13">
+      <c r="A471" s="1" t="s">
+        <v>2791</v>
+      </c>
+      <c r="B471" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C471" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D471" s="1">
+        <v>0</v>
+      </c>
+      <c r="E471" s="1">
+        <v>44</v>
+      </c>
+      <c r="F471" s="1">
+        <v>15</v>
+      </c>
+      <c r="G471" s="1">
+        <v>3</v>
+      </c>
+      <c r="H471" s="1">
+        <v>3</v>
+      </c>
+      <c r="I471" s="1">
+        <v>0</v>
+      </c>
+      <c r="J471" s="1">
+        <v>266</v>
+      </c>
+      <c r="K471" s="1">
+        <v>27</v>
+      </c>
+      <c r="L471" s="1">
+        <v>0.15</v>
+      </c>
+      <c r="M471" s="1">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:Z418" etc:filterBottomFollowUsedRange="0">
     <extLst/>

</xml_diff>